<commit_message>
Fix example rows being parsed as real data during import
- Add "EXAMPLE:" prefix to all example row descriptions in template generator
- Add green fill (E2EFDA) detection in parser to skip example rows
- Update Introduction sheet to note examples are auto-skipped
- Regenerate template file with updated examples

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/climatrix_files/climatrix_scope3_template_v1.xlsx
+++ b/backend/climatrix_files/climatrix_scope3_template_v1.xlsx
@@ -605,7 +605,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Template Version: 1.0 | Generated: 2026-03-01 17:58</t>
+          <t>Template Version: 1.0 | Generated: 2026-03-01 18:26</t>
         </is>
       </c>
     </row>
@@ -915,7 +915,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - GREEN rows: Example data (delete before uploading)</t>
+          <t xml:space="preserve">   - GREEN rows: Example data (auto-skipped during import, or delete them)</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   GREEN row = Example data (for reference, delete before upload)</t>
+          <t xml:space="preserve">   GREEN row = Example data (auto-skipped during import)</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1077,7 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6. Delete the green example row before uploading</t>
+          <t xml:space="preserve">   6. Green example rows are auto-skipped during import (no need to delete)</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>50 laptops for employees</t>
+          <t>EXAMPLE: 50 laptops for employees</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Fleet vehicle purchase</t>
+          <t>EXAMPLE: Fleet vehicle purchase</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -1358,7 +1358,7 @@
       <c r="C8" s="12" t="inlineStr"/>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>CNC machine purchase</t>
+          <t>EXAMPLE: CNC machine purchase</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr"/>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Raw materials from China</t>
+          <t>EXAMPLE: Raw materials from China</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Components from Germany</t>
+          <t>EXAMPLE: Components from Germany</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Urgent parts from US</t>
+          <t>EXAMPLE: Urgent parts from US</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Local delivery (spend)</t>
+          <t>EXAMPLE: Local delivery (spend)</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr"/>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Office paper waste</t>
+          <t>EXAMPLE: Office paper waste</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -3745,7 +3745,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>General office waste</t>
+          <t>EXAMPLE: General office waste</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Waste disposal contract</t>
+          <t>EXAMPLE: Waste disposal contract</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr"/>
@@ -4634,7 +4634,7 @@
       <c r="I7" s="12" t="inlineStr"/>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>John Smith</t>
+          <t>EXAMPLE: John Smith</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
@@ -4683,7 +4683,7 @@
       <c r="I8" s="12" t="inlineStr"/>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>Jane Doe</t>
+          <t>EXAMPLE: Jane Doe</t>
         </is>
       </c>
       <c r="K8" s="12" t="inlineStr">
@@ -4716,7 +4716,7 @@
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Team trip</t>
+          <t>EXAMPLE: Team trip</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -6207,7 +6207,7 @@
       <c r="G6" s="12" t="inlineStr"/>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>John Smith</t>
+          <t>EXAMPLE: John Smith</t>
         </is>
       </c>
       <c r="I6" s="12" t="inlineStr">
@@ -6246,7 +6246,7 @@
       <c r="G7" s="12" t="inlineStr"/>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>EXAMPLE: Team</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>Jane Doe</t>
+          <t>EXAMPLE: Jane Doe</t>
         </is>
       </c>
       <c r="I8" s="12" t="inlineStr">
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>London to Manchester round trip</t>
+          <t>EXAMPLE: London to Manchester round trip</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr"/>
@@ -7009,7 +7009,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Airport transfer</t>
+          <t>EXAMPLE: Airport transfer</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr"/>
@@ -7034,7 +7034,7 @@
       <c r="C8" s="12" t="inlineStr"/>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Weekly rental</t>
+          <t>EXAMPLE: Weekly rental</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -7718,7 +7718,7 @@
       <c r="J6" s="12" t="inlineStr"/>
       <c r="K6" s="12" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>EXAMPLE: R&amp;D</t>
         </is>
       </c>
     </row>
@@ -7767,7 +7767,7 @@
       <c r="J7" s="12" t="inlineStr"/>
       <c r="K7" s="12" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>EXAMPLE: Operations</t>
         </is>
       </c>
     </row>
@@ -7812,7 +7812,7 @@
       <c r="J8" s="12" t="inlineStr"/>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>London Office</t>
+          <t>EXAMPLE: London Office</t>
         </is>
       </c>
     </row>
@@ -7857,7 +7857,7 @@
       <c r="J9" s="12" t="inlineStr"/>
       <c r="K9" s="12" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>EXAMPLE: Support</t>
         </is>
       </c>
     </row>
@@ -7894,7 +7894,7 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>US Subsidiary</t>
+          <t>EXAMPLE: US Subsidiary</t>
         </is>
       </c>
     </row>
@@ -8753,7 +8753,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Leased HQ - Tel Aviv</t>
+          <t>EXAMPLE: Leased HQ - Tel Aviv</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Distribution center</t>
+          <t>EXAMPLE: Distribution center</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
@@ -8849,7 +8849,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Cloud hosting facility</t>
+          <t>EXAMPLE: Cloud hosting facility</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -8899,7 +8899,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Small satellite office</t>
+          <t>EXAMPLE: Small satellite office</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr"/>
@@ -9811,7 +9811,7 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Products to EU market</t>
+          <t>EXAMPLE: Products to EU market</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
@@ -9856,7 +9856,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Local deliveries</t>
+          <t>EXAMPLE: Local deliveries</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr"/>
@@ -10734,7 +10734,7 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Steel plates for auto parts</t>
+          <t>EXAMPLE: Steel plates for auto parts</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
@@ -10767,7 +10767,7 @@
       <c r="D8" s="12" t="inlineStr"/>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Revenue from processed goods</t>
+          <t>EXAMPLE: Revenue from processed goods</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr"/>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Window AC units sold</t>
+          <t>EXAMPLE: Window AC units sold</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -11856,7 +11856,7 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Diesel trucks sold</t>
+          <t>EXAMPLE: Diesel trucks sold</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -12781,7 +12781,7 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Product packaging waste</t>
+          <t>EXAMPLE: Product packaging waste</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
@@ -12822,7 +12822,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>E-waste from sold devices</t>
+          <t>EXAMPLE: E-waste from sold devices</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
@@ -13708,7 +13708,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Leased office space - Floor 3</t>
+          <t>EXAMPLE: Leased office space - Floor 3</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -13763,7 +13763,7 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Leased warehouse</t>
+          <t>EXAMPLE: Leased warehouse</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr"/>
@@ -14762,7 +14762,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Main St. franchise</t>
+          <t>EXAMPLE: Main St. franchise</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -14817,7 +14817,7 @@
       <c r="C8" s="12" t="inlineStr"/>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Mall franchise</t>
+          <t>EXAMPLE: Mall franchise</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr"/>
@@ -16761,7 +16761,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Office heating - Q1 2024</t>
+          <t>EXAMPLE: Office heating - Q1 2024</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -16798,7 +16798,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Backup generator</t>
+          <t>EXAMPLE: Backup generator</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -16835,7 +16835,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Monthly gas bill</t>
+          <t>EXAMPLE: Monthly gas bill</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
@@ -17772,7 +17772,7 @@
       <formula1>"Physical,Spend"</formula1>
     </dataValidation>
     <dataValidation sqref="E6:E108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Please select a valid unit or currency" type="list">
-      <formula1>"m3,kWh,tonnes,kg,liters,USD,EUR,GBP,ILS,AUD,CAD,CHF,CNY,JPY,Other"</formula1>
+      <formula1>"kg,liters,m3,tonnes,kWh,USD,EUR,GBP,ILS,AUD,CAD,CHF,CNY,JPY,Other"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17903,7 +17903,7 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Sales team vehicle ABC-123</t>
+          <t>EXAMPLE: Sales team vehicle ABC-123</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -17940,7 +17940,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Delivery truck fleet</t>
+          <t>EXAMPLE: Delivery truck fleet</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -17977,7 +17977,7 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Fleet fuel purchase</t>
+          <t>EXAMPLE: Fleet fuel purchase</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -18014,7 +18014,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Monthly fuel cards</t>
+          <t>EXAMPLE: Monthly fuel cards</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -19064,7 +19064,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>AC system refill - Building A</t>
+          <t>EXAMPLE: AC system refill - Building A</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -19096,7 +19096,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Refrigerant purchase invoice</t>
+          <t>EXAMPLE: Refrigerant purchase invoice</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -19687,7 +19687,7 @@
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>Main office - Tel Aviv</t>
+          <t>EXAMPLE: Main office - Tel Aviv</t>
         </is>
       </c>
       <c r="G6" s="12" t="inlineStr">
@@ -19730,7 +19730,7 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>US subsidiary</t>
+          <t>EXAMPLE: US subsidiary</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
@@ -19773,7 +19773,7 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>Germany office - bill</t>
+          <t>EXAMPLE: Germany office - bill</t>
         </is>
       </c>
       <c r="G8" s="12" t="inlineStr">
@@ -19820,7 +19820,7 @@
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>IL - OPC power producer</t>
+          <t>EXAMPLE: IL - OPC power producer</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
@@ -19863,7 +19863,7 @@
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>UK - residual mix</t>
+          <t>EXAMPLE: UK - residual mix</t>
         </is>
       </c>
       <c r="G10" s="12" t="inlineStr">
@@ -19906,7 +19906,7 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Data center - RECs</t>
+          <t>EXAMPLE: Data center - RECs</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
@@ -21160,7 +21160,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Office heating - Winter 2024</t>
+          <t>EXAMPLE: Office heating - Winter 2024</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -21192,7 +21192,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Manufacturing process steam</t>
+          <t>EXAMPLE: Manufacturing process steam</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -21224,7 +21224,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Monthly heating bill</t>
+          <t>EXAMPLE: Monthly heating bill</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
@@ -21771,7 +21771,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Data center cooling</t>
+          <t>EXAMPLE: Data center cooling</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -21803,7 +21803,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Office cooling - Summer</t>
+          <t>EXAMPLE: Office cooling - Summer</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -21835,7 +21835,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Monthly cooling bill</t>
+          <t>EXAMPLE: Monthly cooling bill</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
@@ -22426,7 +22426,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Raw steel plates for production</t>
+          <t>EXAMPLE: Raw steel plates for production</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -22466,7 +22466,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Annual office supplies</t>
+          <t>EXAMPLE: Annual office supplies</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr"/>
@@ -22502,7 +22502,7 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>PET bottles from supplier</t>
+          <t>EXAMPLE: PET bottles from supplier</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">

</xml_diff>